<commit_message>
fix: BOQ parser column letter resolution + header row auto-detect
</commit_message>
<xml_diff>
--- a/QS-WFUI-Info.xlsx
+++ b/QS-WFUI-Info.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\00 CIPAA contract work dairy\QS-WFUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E27DE7F8-2F50-4807-B217-86D9B93038A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26318067-13C2-4FA1-99C5-D443DD6BBF1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="38">
   <si>
     <t>MyQSWFUI16071995#</t>
   </si>
@@ -73,14 +74,319 @@
   </si>
   <si>
     <t>"https://fsrdasrwceuscrfglskd.supabase.co</t>
+  </si>
+  <si>
+    <t>Next Plan — Sprint 7, 8, 9, 10</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">To reach a </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>real public demo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, the next 4 sprints should be:</t>
+    </r>
+  </si>
+  <si>
+    <t>Sprint 7 — Real File Upload + BOQ Parser</t>
+  </si>
+  <si>
+    <r>
+      <t>document.upload_file</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → store file in Supabase Storage</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>document.read_excel</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → parse actual .xlsx using a library (e.g. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>xlsx</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>qs.read_boq</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → extract structured BOQ rows from parsed data</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">API endpoint: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>POST /uploads</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> with multipart form</t>
+    </r>
+  </si>
+  <si>
+    <t>Sprint 8 — Real AI Integration</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Wire </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>qs.classify_trade</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to an actual LLM (OpenAI GPT-4o or Claude via API)</t>
+    </r>
+  </si>
+  <si>
+    <t>Return confidence scores per item</t>
+  </si>
+  <si>
+    <t>Vol 11 (AI Governance): prompt versioning, confidence threshold, low-confidence flagging</t>
+  </si>
+  <si>
+    <t>Sprint 9 — Real Document Generation</t>
+  </si>
+  <si>
+    <r>
+      <t>procurement.generate_rfq</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → generate actual </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>.docx</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> RFQ using </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>docxtemplater</t>
+    </r>
+  </si>
+  <si>
+    <t>Store artifact in Supabase Storage</t>
+  </si>
+  <si>
+    <r>
+      <t>document.save_file</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → persists to </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>/artifacts/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> folder</t>
+    </r>
+  </si>
+  <si>
+    <t>Artifact viewer + download button in UI</t>
+  </si>
+  <si>
+    <t>Sprint 10 — Human Approval Flow</t>
+  </si>
+  <si>
+    <r>
+      <t>core.human_approval</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → pauses execution, sends notification</t>
+    </r>
+  </si>
+  <si>
+    <t>Approval screen in UI (list pending approvals, approve/reject)</t>
+  </si>
+  <si>
+    <t>Runner resumes after approval</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">This completes the Vol 0 formula: </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>AI accelerates → Human approves → System records</t>
+    </r>
+  </si>
+  <si>
+    <t>After Sprint 10 you'll have a complete, demo-ready BOQ-to-RFQ workflow — Stage 1 of the roadmap done for real. That's the right moment for the first public demo.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13.5"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -108,11 +414,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -395,7 +711,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:E11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
@@ -403,7 +719,7 @@
     <col min="4" max="4" width="38.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -420,12 +736,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5">
       <c r="B6" t="s">
         <v>5</v>
       </c>
@@ -436,7 +752,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5">
       <c r="B8" t="s">
         <v>6</v>
       </c>
@@ -444,7 +760,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5">
       <c r="B9" t="s">
         <v>7</v>
       </c>
@@ -452,7 +768,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5">
       <c r="B10" t="s">
         <v>8</v>
       </c>
@@ -460,12 +776,147 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5">
       <c r="B11" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C11" t="s">
         <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F797E672-8912-4C15-9F21-5332AC010547}">
+  <dimension ref="B2:B33"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="150.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:2" ht="18">
+      <c r="B2" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="2:2">
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="2:2">
+      <c r="B6" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="2:2">
+      <c r="B7" s="5"/>
+    </row>
+    <row r="8" spans="2:2">
+      <c r="B8" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="2:2">
+      <c r="B9" s="6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="2:2">
+      <c r="B10" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="2:2">
+      <c r="B11" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" spans="2:2">
+      <c r="B13" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="2:2">
+      <c r="B14" s="5"/>
+    </row>
+    <row r="15" spans="2:2">
+      <c r="B15" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="2:2">
+      <c r="B16" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2">
+      <c r="B17" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2">
+      <c r="B19" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2">
+      <c r="B20" s="5"/>
+    </row>
+    <row r="21" spans="2:2">
+      <c r="B21" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="22" spans="2:2">
+      <c r="B22" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="23" spans="2:2">
+      <c r="B23" s="6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="24" spans="2:2">
+      <c r="B24" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="26" spans="2:2">
+      <c r="B26" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="27" spans="2:2">
+      <c r="B27" s="5"/>
+    </row>
+    <row r="28" spans="2:2">
+      <c r="B28" s="6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="29" spans="2:2">
+      <c r="B29" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="30" spans="2:2">
+      <c r="B30" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="31" spans="2:2">
+      <c r="B31" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="33" spans="2:2">
+      <c r="B33" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(runtime): add Phase 27 official pack readiness baseline
- inventory all official packs, nodes, templates, and workflow bodies
- reconcile declared executors with live resolver wiring
- validate graph node, port, and cycle integrity
- generate machine-readable and human-readable readiness reports
- rank runtime, configuration, connector, and template blockers
- complete the S27.0 checklist and handover
</commit_message>
<xml_diff>
--- a/QS-WFUI-Info.xlsx
+++ b/QS-WFUI-Info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\00 CIPAA contract work dairy\QS-WFUI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A096B4D9-8974-49AA-995A-5BCBEB149B2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0E6C721-D46B-4C02-B476-0661848DA013}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
     <sheet name="Sheet4" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="114">
   <si>
     <t>MyQSWFUI16071995#</t>
   </si>
@@ -1183,6 +1183,12 @@
       </rPr>
       <t xml:space="preserve"> — docs/memory close-out</t>
     </r>
+  </si>
+  <si>
+    <t>Railway</t>
+  </si>
+  <si>
+    <t>Login using github</t>
   </si>
 </sst>
 </file>
@@ -1566,7 +1572,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:E30"/>
+  <dimension ref="A2:E34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="32.85546875" bestFit="1" customWidth="1"/>
@@ -1713,6 +1719,14 @@
       </c>
       <c r="C30" t="s">
         <v>49</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" t="s">
+        <v>112</v>
+      </c>
+      <c r="B34" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>